<commit_message>
Record the verified Combine-Harvest row, image, and BLM inventory.
Align the three partial index date displays with the Overtime M/D/YYYY format and add the counted inventory to the reconciliation workbook.

Co-authored-by: rodneydanger84 <rodneydanger84@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/combine_harvest_abstract/deliverables/19-47N-76W/47N-76W-19_Johnson_Co_Penterra_Abstract_Index.xlsx
+++ b/combine_harvest_abstract/deliverables/19-47N-76W/47N-76W-19_Johnson_Co_Penterra_Abstract_Index.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Index" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Qualifications" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Index" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Qualifications" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Index'!$1:$9</definedName>
@@ -101,7 +101,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -158,6 +158,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -615,10 +618,10 @@
           <t>87A35-0318</t>
         </is>
       </c>
-      <c r="F10" s="19" t="n">
+      <c r="F10" s="20" t="n">
         <v>34365</v>
       </c>
-      <c r="G10" s="19" t="n">
+      <c r="G10" s="20" t="n">
         <v>34366</v>
       </c>
       <c r="H10" s="17" t="inlineStr">
@@ -654,10 +657,10 @@
           <t>RW32-0623-0632</t>
         </is>
       </c>
-      <c r="F11" s="19" t="n">
+      <c r="F11" s="20" t="n">
         <v>43087</v>
       </c>
-      <c r="G11" s="19" t="n">
+      <c r="G11" s="20" t="n">
         <v>43210</v>
       </c>
       <c r="H11" s="17" t="inlineStr">

</xml_diff>